<commit_message>
refactor: update funcion names
</commit_message>
<xml_diff>
--- a/src/debug/clean_fato_atividades.xlsx
+++ b/src/debug/clean_fato_atividades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,35 +434,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>coeficiente_de_qualidade_categorizado</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>tem_interesse_em_stem</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>participacao_previa_stem</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>sk_participante</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>sk_evento</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sk_tempo</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>sk_fato_atividade</t>
         </is>
@@ -478,27 +473,22 @@
       <c r="C2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D2" t="b">
+        <v>1</v>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I2" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -512,27 +502,22 @@
       <c r="C3" t="n">
         <v>5</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D3" t="b">
+        <v>1</v>
       </c>
       <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I3" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -546,27 +531,22 @@
       <c r="C4" t="n">
         <v>2.5</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D4" t="b">
+        <v>1</v>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I4" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -580,27 +560,22 @@
       <c r="C5" t="n">
         <v>3.5</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D5" t="b">
+        <v>0</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
-      <c r="F5" t="b">
-        <v>0</v>
+      <c r="F5" t="n">
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I5" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -614,27 +589,22 @@
       <c r="C6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D6" t="b">
+        <v>1</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="F6" t="b">
-        <v>1</v>
+      <c r="F6" t="n">
+        <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I6" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -648,27 +618,22 @@
       <c r="C7" t="n">
         <v>4.5</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D7" t="b">
+        <v>0</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
       </c>
-      <c r="F7" t="b">
-        <v>0</v>
+      <c r="F7" t="n">
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I7" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J7" t="n">
         <v>6</v>
       </c>
     </row>
@@ -682,27 +647,22 @@
       <c r="C8" t="n">
         <v>3.5</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D8" t="b">
+        <v>0</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
       </c>
-      <c r="F8" t="b">
-        <v>0</v>
+      <c r="F8" t="n">
+        <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I8" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J8" t="n">
         <v>7</v>
       </c>
     </row>
@@ -716,27 +676,22 @@
       <c r="C9" t="n">
         <v>4.5</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D9" t="b">
+        <v>1</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
-      <c r="F9" t="b">
-        <v>1</v>
+      <c r="F9" t="n">
+        <v>8</v>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I9" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J9" t="n">
         <v>8</v>
       </c>
     </row>
@@ -750,27 +705,22 @@
       <c r="C10" t="n">
         <v>4</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D10" t="b">
+        <v>1</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
-      <c r="F10" t="b">
-        <v>1</v>
+      <c r="F10" t="n">
+        <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I10" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J10" t="n">
         <v>9</v>
       </c>
     </row>
@@ -784,27 +734,22 @@
       <c r="C11" t="n">
         <v>4</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D11" t="b">
+        <v>0</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
       </c>
-      <c r="F11" t="b">
-        <v>0</v>
+      <c r="F11" t="n">
+        <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I11" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J11" t="n">
         <v>10</v>
       </c>
     </row>
@@ -818,27 +763,22 @@
       <c r="C12" t="n">
         <v>5</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D12" t="b">
+        <v>0</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
       </c>
-      <c r="F12" t="b">
-        <v>0</v>
+      <c r="F12" t="n">
+        <v>11</v>
       </c>
       <c r="G12" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I12" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J12" t="n">
         <v>11</v>
       </c>
     </row>
@@ -852,27 +792,22 @@
       <c r="C13" t="n">
         <v>4.5</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D13" t="b">
+        <v>1</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
       </c>
-      <c r="F13" t="b">
-        <v>1</v>
+      <c r="F13" t="n">
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>20240611</v>
       </c>
       <c r="I13" t="n">
-        <v>20240611</v>
-      </c>
-      <c r="J13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -886,27 +821,22 @@
       <c r="C14" t="n">
         <v>3.5</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D14" t="b">
+        <v>0</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
       </c>
-      <c r="F14" t="b">
-        <v>0</v>
+      <c r="F14" t="n">
+        <v>13</v>
       </c>
       <c r="G14" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I14" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J14" t="n">
         <v>13</v>
       </c>
     </row>
@@ -920,27 +850,22 @@
       <c r="C15" t="n">
         <v>5</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D15" t="b">
+        <v>0</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
       </c>
-      <c r="F15" t="b">
-        <v>0</v>
+      <c r="F15" t="n">
+        <v>14</v>
       </c>
       <c r="G15" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I15" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -954,27 +879,22 @@
       <c r="C16" t="n">
         <v>3</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D16" t="b">
+        <v>1</v>
       </c>
       <c r="E16" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>15</v>
       </c>
       <c r="G16" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I16" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -988,27 +908,22 @@
       <c r="C17" t="n">
         <v>4</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D17" t="b">
+        <v>1</v>
       </c>
       <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>16</v>
       </c>
       <c r="G17" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I17" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1022,27 +937,22 @@
       <c r="C18" t="n">
         <v>4</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D18" t="b">
+        <v>1</v>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17</v>
       </c>
       <c r="G18" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I18" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J18" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1056,27 +966,22 @@
       <c r="C19" t="n">
         <v>2.5</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D19" t="b">
+        <v>0</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
       </c>
-      <c r="F19" t="b">
-        <v>0</v>
+      <c r="F19" t="n">
+        <v>18</v>
       </c>
       <c r="G19" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I19" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J19" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1090,27 +995,22 @@
       <c r="C20" t="n">
         <v>4</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D20" t="b">
+        <v>0</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
       </c>
-      <c r="F20" t="b">
-        <v>0</v>
+      <c r="F20" t="n">
+        <v>19</v>
       </c>
       <c r="G20" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I20" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J20" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1124,27 +1024,22 @@
       <c r="C21" t="n">
         <v>3.5</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D21" t="b">
+        <v>0</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
       </c>
-      <c r="F21" t="b">
-        <v>0</v>
+      <c r="F21" t="n">
+        <v>20</v>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I21" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J21" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1158,27 +1053,22 @@
       <c r="C22" t="n">
         <v>3.5</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D22" t="b">
+        <v>1</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
       </c>
-      <c r="F22" t="b">
-        <v>1</v>
+      <c r="F22" t="n">
+        <v>21</v>
       </c>
       <c r="G22" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I22" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J22" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1192,27 +1082,22 @@
       <c r="C23" t="n">
         <v>3</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D23" t="b">
+        <v>1</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
       </c>
-      <c r="F23" t="b">
-        <v>1</v>
+      <c r="F23" t="n">
+        <v>22</v>
       </c>
       <c r="G23" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I23" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1226,27 +1111,22 @@
       <c r="C24" t="n">
         <v>3.5</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D24" t="b">
+        <v>0</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
       </c>
-      <c r="F24" t="b">
-        <v>0</v>
+      <c r="F24" t="n">
+        <v>23</v>
       </c>
       <c r="G24" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I24" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J24" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1260,27 +1140,22 @@
       <c r="C25" t="n">
         <v>4.5</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D25" t="b">
+        <v>1</v>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
-      </c>
-      <c r="F25" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>24</v>
       </c>
       <c r="G25" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I25" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J25" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1294,27 +1169,22 @@
       <c r="C26" t="n">
         <v>3</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D26" t="b">
+        <v>0</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
       </c>
-      <c r="F26" t="b">
-        <v>0</v>
+      <c r="F26" t="n">
+        <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I26" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J26" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1328,27 +1198,22 @@
       <c r="C27" t="n">
         <v>3.5</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D27" t="b">
+        <v>0</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
       </c>
-      <c r="F27" t="b">
-        <v>0</v>
+      <c r="F27" t="n">
+        <v>26</v>
       </c>
       <c r="G27" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I27" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J27" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1362,27 +1227,22 @@
       <c r="C28" t="n">
         <v>4</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D28" t="b">
+        <v>1</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
       </c>
-      <c r="F28" t="b">
-        <v>1</v>
+      <c r="F28" t="n">
+        <v>27</v>
       </c>
       <c r="G28" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I28" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J28" t="n">
         <v>27</v>
       </c>
     </row>
@@ -1396,27 +1256,22 @@
       <c r="C29" t="n">
         <v>4.5</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D29" t="b">
+        <v>1</v>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
-      </c>
-      <c r="F29" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>28</v>
       </c>
       <c r="G29" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>20240613</v>
       </c>
       <c r="I29" t="n">
-        <v>20240613</v>
-      </c>
-      <c r="J29" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1430,27 +1285,22 @@
       <c r="C30" t="n">
         <v>4.5</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D30" t="b">
+        <v>0</v>
       </c>
       <c r="E30" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>29</v>
       </c>
       <c r="G30" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>20241031</v>
       </c>
       <c r="I30" t="n">
-        <v>20241031</v>
-      </c>
-      <c r="J30" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1464,27 +1314,22 @@
       <c r="C31" t="n">
         <v>4</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D31" t="b">
+        <v>1</v>
       </c>
       <c r="E31" t="b">
-        <v>1</v>
-      </c>
-      <c r="F31" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>30</v>
       </c>
       <c r="G31" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I31" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J31" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1498,27 +1343,22 @@
       <c r="C32" t="n">
         <v>5</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D32" t="b">
+        <v>1</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
       </c>
-      <c r="F32" t="b">
-        <v>1</v>
+      <c r="F32" t="n">
+        <v>31</v>
       </c>
       <c r="G32" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="H32" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I32" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J32" t="n">
         <v>31</v>
       </c>
     </row>
@@ -1532,27 +1372,22 @@
       <c r="C33" t="n">
         <v>4</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D33" t="b">
+        <v>0</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
       </c>
-      <c r="F33" t="b">
-        <v>0</v>
+      <c r="F33" t="n">
+        <v>32</v>
       </c>
       <c r="G33" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I33" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J33" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1566,27 +1401,22 @@
       <c r="C34" t="n">
         <v>5</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D34" t="b">
+        <v>0</v>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F34" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>33</v>
       </c>
       <c r="G34" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I34" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J34" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1600,27 +1430,22 @@
       <c r="C35" t="n">
         <v>3.5</v>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D35" t="b">
+        <v>0</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
       </c>
-      <c r="F35" t="b">
-        <v>0</v>
+      <c r="F35" t="n">
+        <v>34</v>
       </c>
       <c r="G35" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="H35" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I35" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J35" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1634,27 +1459,22 @@
       <c r="C36" t="n">
         <v>2.5</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
+      <c r="D36" t="b">
+        <v>0</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
       </c>
-      <c r="F36" t="b">
-        <v>0</v>
+      <c r="F36" t="n">
+        <v>35</v>
       </c>
       <c r="G36" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I36" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J36" t="n">
         <v>35</v>
       </c>
     </row>
@@ -1668,27 +1488,22 @@
       <c r="C37" t="n">
         <v>4</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D37" t="b">
+        <v>0</v>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
-      </c>
-      <c r="F37" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>36</v>
       </c>
       <c r="G37" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>20250313</v>
       </c>
       <c r="I37" t="n">
-        <v>20250313</v>
-      </c>
-      <c r="J37" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1702,27 +1517,22 @@
       <c r="C38" t="n">
         <v>5</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D38" t="b">
+        <v>1</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
       </c>
-      <c r="F38" t="b">
-        <v>1</v>
+      <c r="F38" t="n">
+        <v>37</v>
       </c>
       <c r="G38" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>20250318</v>
       </c>
       <c r="I38" t="n">
-        <v>20250318</v>
-      </c>
-      <c r="J38" t="n">
         <v>37</v>
       </c>
     </row>
@@ -1736,27 +1546,22 @@
       <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D39" t="b">
+        <v>0</v>
       </c>
       <c r="E39" t="b">
-        <v>0</v>
-      </c>
-      <c r="F39" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>38</v>
       </c>
       <c r="G39" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>20250318</v>
       </c>
       <c r="I39" t="n">
-        <v>20250318</v>
-      </c>
-      <c r="J39" t="n">
         <v>38</v>
       </c>
     </row>
@@ -1770,27 +1575,22 @@
       <c r="C40" t="n">
         <v>5</v>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Muito alto</t>
-        </is>
+      <c r="D40" t="b">
+        <v>1</v>
       </c>
       <c r="E40" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" t="b">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>39</v>
       </c>
       <c r="G40" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>20250318</v>
       </c>
       <c r="I40" t="n">
-        <v>20250318</v>
-      </c>
-      <c r="J40" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1804,27 +1604,22 @@
       <c r="C41" t="n">
         <v>4</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D41" t="b">
+        <v>0</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
       </c>
-      <c r="F41" t="b">
-        <v>0</v>
+      <c r="F41" t="n">
+        <v>40</v>
       </c>
       <c r="G41" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="H41" t="n">
-        <v>5</v>
+        <v>20250318</v>
       </c>
       <c r="I41" t="n">
-        <v>20250318</v>
-      </c>
-      <c r="J41" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1838,27 +1633,22 @@
       <c r="C42" t="n">
         <v>3.5</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
+      <c r="D42" t="b">
+        <v>0</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
       </c>
-      <c r="F42" t="b">
-        <v>0</v>
+      <c r="F42" t="n">
+        <v>41</v>
       </c>
       <c r="G42" t="n">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>20250318</v>
       </c>
       <c r="I42" t="n">
-        <v>20250318</v>
-      </c>
-      <c r="J42" t="n">
         <v>41</v>
       </c>
     </row>

</xml_diff>